<commit_message>
Fix: Google Drive uploader log guidance and quarterly financial statements parsing and integration
</commit_message>
<xml_diff>
--- a/Bao cao/TCB/TCB_Model_2026-06.xlsx
+++ b/Bao cao/TCB/TCB_Model_2026-06.xlsx
@@ -1,14 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P&amp;L" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="01_Cover" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="02_Assumptions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="04_PnL" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="06_Ratios" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +19,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="#,##0.0"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -27,14 +32,16 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Segoe UI"/>
       <b val="1"/>
-      <sz val="18"/>
+      <color rgb="001A365D"/>
+      <sz val="16"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Segoe UI"/>
       <i val="1"/>
-      <sz val="12"/>
+      <color rgb="004A5568"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
@@ -57,11 +64,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -427,41 +438,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:B6"/>
+  <dimension ref="B2:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>BÁO CÁO PHÂN TÍCH CỔ PHIẾU TCB</t>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>MÔ HÌNH PHÂN TÍCH TÀI CHÍNH &amp; ĐỊNH GIÁ TCB</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Vietnam Technological And Commercial Joint Stock Bank</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Giá hiện tại:</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>33400</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Vốn hóa (tỷ):</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>236680.4298276</v>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Ngân hàng Thương mại Cổ phần Kỹ thương Việt Nam</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -475,13 +466,89 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Giả định</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Giá trị</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Chi phí vốn (COE)</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>0.112</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tốc độ tăng trưởng dài hạn (g)</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>P/B Mục tiêu</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Tín dụng tăng trưởng (F)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Huy động tăng trưởng (F)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0.16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Chỉ tiêu</t>
+          <t>Chỉ tiêu P&amp;L (tỷ VND)</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -528,125 +595,372 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Doanh thu thuần (tỷ)</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" s="3" t="n">
-        <v>0</v>
+          <t>Thu nhập lãi thuần (NII)</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>26698.613</v>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>30289.775</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>27691.12</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>35507.963</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>38155.091</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>37023.55918905001</v>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>43525.010266311</v>
+      </c>
+      <c r="I2" s="5" t="n">
+        <v>51170.67620519609</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Lợi nhuận gộp (tỷ)</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="3" t="n">
-        <v>0</v>
+          <t>Lợi nhuận sau thuế (LNST)</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>18052.25</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>20150.377</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>18003.802</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>21522.928</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>25290.23</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>28320.48953020379</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>32460.56976129289</v>
+      </c>
+      <c r="I3" s="5" t="n">
+        <v>37262.35915118305</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lợi nhuận sau thuế (tỷ)</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>18052.25</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>20150.377</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>18003.802</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>21522.928</v>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>25290.23</v>
-      </c>
-      <c r="G4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="3" t="n">
-        <v>0</v>
+          <t>EPS (VND)</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>5137</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>5725</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>2549</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>3049</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>3572</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>3996.546536891945</v>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>4580.788673397658</v>
+      </c>
+      <c r="I4" s="6" t="n">
+        <v>5258.410249697858</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>EPS (VND)</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>5137</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>5725</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>2549</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>3049</v>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>3572</v>
-      </c>
-      <c r="G5" s="3" t="n">
+          <t>Vốn chủ sở hữu (VCSH)</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>93041.47199999999</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>113424.966</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>131616.065</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>147939.621</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>179501.442</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>203573.8581006732</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>231165.3423977722</v>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>262838.3476762778</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Chỉ số tài chính</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>2021A</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>2022A</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>2023A</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>2024A</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>2025A</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>2026E</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>2027E</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>2028E</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>NIM (%)</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>0.0469</v>
+      </c>
+      <c r="C2" s="7" t="n">
+        <v>0.0433</v>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>0.0326</v>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>0.0363</v>
+      </c>
+      <c r="F2" s="7" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>0.0277</v>
+      </c>
+      <c r="H2" s="7" t="n">
+        <v>0.0291</v>
+      </c>
+      <c r="I2" s="7" t="n">
+        <v>0.0305</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ROE (%)</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>0.194</v>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>0.1777</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>0.1368</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>0.1455</v>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>0.1409</v>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>0.1391</v>
+      </c>
+      <c r="H3" s="7" t="n">
+        <v>0.1404</v>
+      </c>
+      <c r="I3" s="7" t="n">
+        <v>0.1418</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ROA (%)</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>0.0317</v>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>0.0288</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>0.0212</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>0.0212</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>0.0212</v>
+      </c>
+      <c r="H4" s="7" t="n">
+        <v>0.0217</v>
+      </c>
+      <c r="I4" s="7" t="n">
+        <v>0.0222</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>LDR (%)</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>0.9861</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>1.0595</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>0.9502</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>0.9255</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>0.9076</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>0.9232</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>0.9391</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>0.9553</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CASA (%)</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="3" t="n">
+      <c r="C6" s="7" t="n">
+        <v>0.0052</v>
+      </c>
+      <c r="D6" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="I5" s="3" t="n">
-        <v>0</v>
+      <c r="E6" s="7" t="n">
+        <v>0.0017</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>0.0039</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Tỷ lệ nợ xấu NPL (%)</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>-0.0109</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>-0.0115</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>-0.012</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>-0.013</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>-0.0139</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>0.012</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add quarterly Credit & Funding Growth Chart (32 quarters), fix YTD growth calculation errors, and update Web Dashboard
</commit_message>
<xml_diff>
--- a/Bao cao/TCB/TCB_Model_2026-06.xlsx
+++ b/Bao cao/TCB/TCB_Model_2026-06.xlsx
@@ -24,6 +24,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Investment_Thesis" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Summary_Snapshot" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_PE_PB_History" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Credit_Funding_Growth" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -141,7 +142,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -181,6 +182,8 @@
     <xf numFmtId="167" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2751,6 +2754,662 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Quý</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>Tổng Tín dụng (tỷ VND)</t>
+        </is>
+      </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>Tổng Huy động (tỷ VND)</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>Tăng trưởng Tín dụng YTD (%)</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>Tăng trưởng Huy động YTD (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="28" t="inlineStr">
+        <is>
+          <t>Q2/18</t>
+        </is>
+      </c>
+      <c r="B2" s="29" t="n">
+        <v>164180.966</v>
+      </c>
+      <c r="C2" s="29" t="n">
+        <v>205187.505</v>
+      </c>
+      <c r="D2" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>Q3/18</t>
+        </is>
+      </c>
+      <c r="B3" s="29" t="n">
+        <v>164282.01</v>
+      </c>
+      <c r="C3" s="29" t="n">
+        <v>210823.197</v>
+      </c>
+      <c r="D3" s="30" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="E3" s="30" t="n">
+        <v>0.0275</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="28" t="inlineStr">
+        <is>
+          <t>Q4/18</t>
+        </is>
+      </c>
+      <c r="B4" s="29" t="n">
+        <v>157556.934</v>
+      </c>
+      <c r="C4" s="29" t="n">
+        <v>214649.295</v>
+      </c>
+      <c r="D4" s="30" t="n">
+        <v>-0.0403</v>
+      </c>
+      <c r="E4" s="30" t="n">
+        <v>0.0461</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t>Q1/19</t>
+        </is>
+      </c>
+      <c r="B5" s="29" t="n">
+        <v>161272.479</v>
+      </c>
+      <c r="C5" s="29" t="n">
+        <v>220844.216</v>
+      </c>
+      <c r="D5" s="30" t="n">
+        <v>0.0236</v>
+      </c>
+      <c r="E5" s="30" t="n">
+        <v>0.0289</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="28" t="inlineStr">
+        <is>
+          <t>Q2/19</t>
+        </is>
+      </c>
+      <c r="B6" s="29" t="n">
+        <v>182887.287</v>
+      </c>
+      <c r="C6" s="29" t="n">
+        <v>232904.78</v>
+      </c>
+      <c r="D6" s="30" t="n">
+        <v>0.1608</v>
+      </c>
+      <c r="E6" s="30" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>Q3/19</t>
+        </is>
+      </c>
+      <c r="B7" s="29" t="n">
+        <v>202462.011</v>
+      </c>
+      <c r="C7" s="29" t="n">
+        <v>233143.291</v>
+      </c>
+      <c r="D7" s="30" t="n">
+        <v>0.285</v>
+      </c>
+      <c r="E7" s="30" t="n">
+        <v>0.0862</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="28" t="inlineStr">
+        <is>
+          <t>Q4/19</t>
+        </is>
+      </c>
+      <c r="B8" s="29" t="n">
+        <v>227885.283</v>
+      </c>
+      <c r="C8" s="29" t="n">
+        <v>248757.395</v>
+      </c>
+      <c r="D8" s="30" t="n">
+        <v>0.4464</v>
+      </c>
+      <c r="E8" s="30" t="n">
+        <v>0.1589</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="28" t="inlineStr">
+        <is>
+          <t>Q1/20</t>
+        </is>
+      </c>
+      <c r="B9" s="29" t="n">
+        <v>229037.642</v>
+      </c>
+      <c r="C9" s="29" t="n">
+        <v>252570.894</v>
+      </c>
+      <c r="D9" s="30" t="n">
+        <v>0.0051</v>
+      </c>
+      <c r="E9" s="30" t="n">
+        <v>0.0153</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="28" t="inlineStr">
+        <is>
+          <t>Q2/20</t>
+        </is>
+      </c>
+      <c r="B10" s="29" t="n">
+        <v>229385.47</v>
+      </c>
+      <c r="C10" s="29" t="n">
+        <v>273261.751</v>
+      </c>
+      <c r="D10" s="30" t="n">
+        <v>0.0066</v>
+      </c>
+      <c r="E10" s="30" t="n">
+        <v>0.09849999999999999</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="28" t="inlineStr">
+        <is>
+          <t>Q3/20</t>
+        </is>
+      </c>
+      <c r="B11" s="29" t="n">
+        <v>228667.892</v>
+      </c>
+      <c r="C11" s="29" t="n">
+        <v>275357.326</v>
+      </c>
+      <c r="D11" s="30" t="n">
+        <v>0.0034</v>
+      </c>
+      <c r="E11" s="30" t="n">
+        <v>0.1069</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="28" t="inlineStr">
+        <is>
+          <t>Q4/20</t>
+        </is>
+      </c>
+      <c r="B12" s="29" t="n">
+        <v>275310.367</v>
+      </c>
+      <c r="C12" s="29" t="n">
+        <v>305358.291</v>
+      </c>
+      <c r="D12" s="30" t="n">
+        <v>0.2081</v>
+      </c>
+      <c r="E12" s="30" t="n">
+        <v>0.2275</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="28" t="inlineStr">
+        <is>
+          <t>Q1/21</t>
+        </is>
+      </c>
+      <c r="B13" s="29" t="n">
+        <v>293799.393</v>
+      </c>
+      <c r="C13" s="29" t="n">
+        <v>313481.366</v>
+      </c>
+      <c r="D13" s="30" t="n">
+        <v>0.0672</v>
+      </c>
+      <c r="E13" s="30" t="n">
+        <v>0.0266</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="28" t="inlineStr">
+        <is>
+          <t>Q2/21</t>
+        </is>
+      </c>
+      <c r="B14" s="29" t="n">
+        <v>310617.819</v>
+      </c>
+      <c r="C14" s="29" t="n">
+        <v>317012.396</v>
+      </c>
+      <c r="D14" s="30" t="n">
+        <v>0.1282</v>
+      </c>
+      <c r="E14" s="30" t="n">
+        <v>0.0382</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="28" t="inlineStr">
+        <is>
+          <t>Q3/21</t>
+        </is>
+      </c>
+      <c r="B15" s="29" t="n">
+        <v>317668.922</v>
+      </c>
+      <c r="C15" s="29" t="n">
+        <v>350378.727</v>
+      </c>
+      <c r="D15" s="30" t="n">
+        <v>0.1539</v>
+      </c>
+      <c r="E15" s="30" t="n">
+        <v>0.1474</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="28" t="inlineStr">
+        <is>
+          <t>Q4/21</t>
+        </is>
+      </c>
+      <c r="B16" s="29" t="n">
+        <v>343605.581</v>
+      </c>
+      <c r="C16" s="29" t="n">
+        <v>348432.349</v>
+      </c>
+      <c r="D16" s="30" t="n">
+        <v>0.2481</v>
+      </c>
+      <c r="E16" s="30" t="n">
+        <v>0.1411</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="28" t="inlineStr">
+        <is>
+          <t>Q1/22</t>
+        </is>
+      </c>
+      <c r="B17" s="29" t="n">
+        <v>361815.215</v>
+      </c>
+      <c r="C17" s="29" t="n">
+        <v>361644.71</v>
+      </c>
+      <c r="D17" s="30" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="E17" s="30" t="n">
+        <v>0.0379</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="28" t="inlineStr">
+        <is>
+          <t>Q2/22</t>
+        </is>
+      </c>
+      <c r="B18" s="29" t="n">
+        <v>387775.129</v>
+      </c>
+      <c r="C18" s="29" t="n">
+        <v>358755.982</v>
+      </c>
+      <c r="D18" s="30" t="n">
+        <v>0.1285</v>
+      </c>
+      <c r="E18" s="30" t="n">
+        <v>0.0296</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="28" t="inlineStr">
+        <is>
+          <t>Q3/22</t>
+        </is>
+      </c>
+      <c r="B19" s="29" t="n">
+        <v>406148.421</v>
+      </c>
+      <c r="C19" s="29" t="n">
+        <v>361776.9</v>
+      </c>
+      <c r="D19" s="30" t="n">
+        <v>0.182</v>
+      </c>
+      <c r="E19" s="30" t="n">
+        <v>0.0383</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="28" t="inlineStr">
+        <is>
+          <t>Q4/22</t>
+        </is>
+      </c>
+      <c r="B20" s="29" t="n">
+        <v>415752.256</v>
+      </c>
+      <c r="C20" s="29" t="n">
+        <v>392410.404</v>
+      </c>
+      <c r="D20" s="30" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="E20" s="30" t="n">
+        <v>0.1262</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="28" t="inlineStr">
+        <is>
+          <t>Q1/23</t>
+        </is>
+      </c>
+      <c r="B21" s="29" t="n">
+        <v>460145.233</v>
+      </c>
+      <c r="C21" s="29" t="n">
+        <v>458633.44595</v>
+      </c>
+      <c r="D21" s="30" t="n">
+        <v>0.1068</v>
+      </c>
+      <c r="E21" s="30" t="n">
+        <v>0.1688</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="28" t="inlineStr">
+        <is>
+          <t>Q2/23</t>
+        </is>
+      </c>
+      <c r="B22" s="29" t="n">
+        <v>460753.044</v>
+      </c>
+      <c r="C22" s="29" t="n">
+        <v>460661.7626</v>
+      </c>
+      <c r="D22" s="30" t="n">
+        <v>0.1082</v>
+      </c>
+      <c r="E22" s="30" t="n">
+        <v>0.1739</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="28" t="inlineStr">
+        <is>
+          <t>Q3/23</t>
+        </is>
+      </c>
+      <c r="B23" s="29" t="n">
+        <v>469588.515</v>
+      </c>
+      <c r="C23" s="29" t="n">
+        <v>496063.26375</v>
+      </c>
+      <c r="D23" s="30" t="n">
+        <v>0.1295</v>
+      </c>
+      <c r="E23" s="30" t="n">
+        <v>0.2641</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="28" t="inlineStr">
+        <is>
+          <t>Q4/23</t>
+        </is>
+      </c>
+      <c r="B24" s="29" t="n">
+        <v>512513.672</v>
+      </c>
+      <c r="C24" s="29" t="n">
+        <v>567554.2774</v>
+      </c>
+      <c r="D24" s="30" t="n">
+        <v>0.2327</v>
+      </c>
+      <c r="E24" s="30" t="n">
+        <v>0.4463</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="28" t="inlineStr">
+        <is>
+          <t>Q1/24</t>
+        </is>
+      </c>
+      <c r="B25" s="29" t="n">
+        <v>552577.121</v>
+      </c>
+      <c r="C25" s="29" t="n">
+        <v>588555.681</v>
+      </c>
+      <c r="D25" s="30" t="n">
+        <v>0.07820000000000001</v>
+      </c>
+      <c r="E25" s="30" t="n">
+        <v>0.03700000000000001</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="28" t="inlineStr">
+        <is>
+          <t>Q2/24</t>
+        </is>
+      </c>
+      <c r="B26" s="29" t="n">
+        <v>584713.478</v>
+      </c>
+      <c r="C26" s="29" t="n">
+        <v>629851.1385</v>
+      </c>
+      <c r="D26" s="30" t="n">
+        <v>0.1409</v>
+      </c>
+      <c r="E26" s="30" t="n">
+        <v>0.1098</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="28" t="inlineStr">
+        <is>
+          <t>Q3/24</t>
+        </is>
+      </c>
+      <c r="B27" s="29" t="n">
+        <v>617924.5699999999</v>
+      </c>
+      <c r="C27" s="29" t="n">
+        <v>646939.245</v>
+      </c>
+      <c r="D27" s="30" t="n">
+        <v>0.2057</v>
+      </c>
+      <c r="E27" s="30" t="n">
+        <v>0.1399</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="28" t="inlineStr">
+        <is>
+          <t>Q4/24</t>
+        </is>
+      </c>
+      <c r="B28" s="29" t="n">
+        <v>623634.2709999999</v>
+      </c>
+      <c r="C28" s="29" t="n">
+        <v>693564.9534999999</v>
+      </c>
+      <c r="D28" s="30" t="n">
+        <v>0.2168</v>
+      </c>
+      <c r="E28" s="30" t="n">
+        <v>0.222</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="28" t="inlineStr">
+        <is>
+          <t>Q1/25</t>
+        </is>
+      </c>
+      <c r="B29" s="29" t="n">
+        <v>655007.208</v>
+      </c>
+      <c r="C29" s="29" t="n">
+        <v>705856.914</v>
+      </c>
+      <c r="D29" s="30" t="n">
+        <v>0.0503</v>
+      </c>
+      <c r="E29" s="30" t="n">
+        <v>0.0177</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="28" t="inlineStr">
+        <is>
+          <t>Q2/25</t>
+        </is>
+      </c>
+      <c r="B30" s="29" t="n">
+        <v>700801.926</v>
+      </c>
+      <c r="C30" s="29" t="n">
+        <v>739872.9861999999</v>
+      </c>
+      <c r="D30" s="30" t="n">
+        <v>0.1237</v>
+      </c>
+      <c r="E30" s="30" t="n">
+        <v>0.0668</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="28" t="inlineStr">
+        <is>
+          <t>Q3/25</t>
+        </is>
+      </c>
+      <c r="B31" s="29" t="n">
+        <v>756078.003</v>
+      </c>
+      <c r="C31" s="29" t="n">
+        <v>801598.9116000001</v>
+      </c>
+      <c r="D31" s="30" t="n">
+        <v>0.2124</v>
+      </c>
+      <c r="E31" s="30" t="n">
+        <v>0.1558</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="28" t="inlineStr">
+        <is>
+          <t>Q4/25</t>
+        </is>
+      </c>
+      <c r="B32" s="29" t="n">
+        <v>757118.751</v>
+      </c>
+      <c r="C32" s="29" t="n">
+        <v>875042.3212</v>
+      </c>
+      <c r="D32" s="30" t="n">
+        <v>0.214</v>
+      </c>
+      <c r="E32" s="30" t="n">
+        <v>0.2617</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="28" t="inlineStr">
+        <is>
+          <t>Q1/26</t>
+        </is>
+      </c>
+      <c r="B33" s="29" t="n">
+        <v>785612.53</v>
+      </c>
+      <c r="C33" s="29" t="n">
+        <v>867468.6972000001</v>
+      </c>
+      <c r="D33" s="30" t="n">
+        <v>0.03759999999999999</v>
+      </c>
+      <c r="E33" s="30" t="n">
+        <v>-0.008699999999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Fix Credit YTD growth calculation by replacing buggy Vietcap NOTES account (nob47/nob48) with correct Balance Sheet corporate bond account (bsb108)
</commit_message>
<xml_diff>
--- a/Bao cao/TCB/TCB_Model_2026-06.xlsx
+++ b/Bao cao/TCB/TCB_Model_2026-06.xlsx
@@ -2047,19 +2047,19 @@
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>93573.522</v>
+        <v>200</v>
       </c>
       <c r="C9" s="13" t="n">
-        <v>79300.508</v>
+        <v>0</v>
       </c>
       <c r="D9" s="13" t="n">
-        <v>118208.799</v>
+        <v>0</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>85211.565</v>
+        <v>6900</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>97010.931</v>
+        <v>0</v>
       </c>
       <c r="G9" s="10" t="n"/>
       <c r="H9" s="10" t="n"/>
@@ -2804,7 +2804,7 @@
         </is>
       </c>
       <c r="B2" s="29" t="n">
-        <v>164180.966</v>
+        <v>168352.166</v>
       </c>
       <c r="C2" s="29" t="n">
         <v>205187.505</v>
@@ -2823,13 +2823,13 @@
         </is>
       </c>
       <c r="B3" s="29" t="n">
-        <v>164282.01</v>
+        <v>180268.21</v>
       </c>
       <c r="C3" s="29" t="n">
         <v>210823.197</v>
       </c>
       <c r="D3" s="30" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0708</v>
       </c>
       <c r="E3" s="30" t="n">
         <v>0.0275</v>
@@ -2842,13 +2842,13 @@
         </is>
       </c>
       <c r="B4" s="29" t="n">
-        <v>157556.934</v>
+        <v>177793.134</v>
       </c>
       <c r="C4" s="29" t="n">
         <v>214649.295</v>
       </c>
       <c r="D4" s="30" t="n">
-        <v>-0.0403</v>
+        <v>0.0561</v>
       </c>
       <c r="E4" s="30" t="n">
         <v>0.0461</v>
@@ -2861,13 +2861,13 @@
         </is>
       </c>
       <c r="B5" s="29" t="n">
-        <v>161272.479</v>
+        <v>177078.679</v>
       </c>
       <c r="C5" s="29" t="n">
         <v>220844.216</v>
       </c>
       <c r="D5" s="30" t="n">
-        <v>0.0236</v>
+        <v>-0.004</v>
       </c>
       <c r="E5" s="30" t="n">
         <v>0.0289</v>
@@ -2880,13 +2880,13 @@
         </is>
       </c>
       <c r="B6" s="29" t="n">
-        <v>182887.287</v>
+        <v>197293.487</v>
       </c>
       <c r="C6" s="29" t="n">
         <v>232904.78</v>
       </c>
       <c r="D6" s="30" t="n">
-        <v>0.1608</v>
+        <v>0.1097</v>
       </c>
       <c r="E6" s="30" t="n">
         <v>0.08500000000000001</v>
@@ -2899,13 +2899,13 @@
         </is>
       </c>
       <c r="B7" s="29" t="n">
-        <v>202462.011</v>
+        <v>211168.211</v>
       </c>
       <c r="C7" s="29" t="n">
         <v>233143.291</v>
       </c>
       <c r="D7" s="30" t="n">
-        <v>0.285</v>
+        <v>0.1877</v>
       </c>
       <c r="E7" s="30" t="n">
         <v>0.0862</v>
@@ -2918,13 +2918,13 @@
         </is>
       </c>
       <c r="B8" s="29" t="n">
-        <v>227885.283</v>
+        <v>228087.289</v>
       </c>
       <c r="C8" s="29" t="n">
         <v>248757.395</v>
       </c>
       <c r="D8" s="30" t="n">
-        <v>0.4464</v>
+        <v>0.2829</v>
       </c>
       <c r="E8" s="30" t="n">
         <v>0.1589</v>
@@ -2937,13 +2937,13 @@
         </is>
       </c>
       <c r="B9" s="29" t="n">
-        <v>229037.642</v>
+        <v>229737.642</v>
       </c>
       <c r="C9" s="29" t="n">
         <v>252570.894</v>
       </c>
       <c r="D9" s="30" t="n">
-        <v>0.0051</v>
+        <v>0.0072</v>
       </c>
       <c r="E9" s="30" t="n">
         <v>0.0153</v>
@@ -2956,13 +2956,13 @@
         </is>
       </c>
       <c r="B10" s="29" t="n">
-        <v>229385.47</v>
+        <v>230085.47</v>
       </c>
       <c r="C10" s="29" t="n">
         <v>273261.751</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>0.0066</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="E10" s="30" t="n">
         <v>0.09849999999999999</v>
@@ -2975,7 +2975,7 @@
         </is>
       </c>
       <c r="B11" s="29" t="n">
-        <v>228667.892</v>
+        <v>228867.892</v>
       </c>
       <c r="C11" s="29" t="n">
         <v>275357.326</v>
@@ -2994,13 +2994,13 @@
         </is>
       </c>
       <c r="B12" s="29" t="n">
-        <v>275310.367</v>
+        <v>275510.367</v>
       </c>
       <c r="C12" s="29" t="n">
         <v>305358.291</v>
       </c>
       <c r="D12" s="30" t="n">
-        <v>0.2081</v>
+        <v>0.2079</v>
       </c>
       <c r="E12" s="30" t="n">
         <v>0.2275</v>
@@ -3013,13 +3013,13 @@
         </is>
       </c>
       <c r="B13" s="29" t="n">
-        <v>293799.393</v>
+        <v>293999.393</v>
       </c>
       <c r="C13" s="29" t="n">
         <v>313481.366</v>
       </c>
       <c r="D13" s="30" t="n">
-        <v>0.0672</v>
+        <v>0.06709999999999999</v>
       </c>
       <c r="E13" s="30" t="n">
         <v>0.0266</v>
@@ -3032,7 +3032,7 @@
         </is>
       </c>
       <c r="B14" s="29" t="n">
-        <v>310617.819</v>
+        <v>310817.819</v>
       </c>
       <c r="C14" s="29" t="n">
         <v>317012.396</v>
@@ -3051,13 +3051,13 @@
         </is>
       </c>
       <c r="B15" s="29" t="n">
-        <v>317668.922</v>
+        <v>317868.922</v>
       </c>
       <c r="C15" s="29" t="n">
         <v>350378.727</v>
       </c>
       <c r="D15" s="30" t="n">
-        <v>0.1539</v>
+        <v>0.1537</v>
       </c>
       <c r="E15" s="30" t="n">
         <v>0.1474</v>
@@ -3070,13 +3070,13 @@
         </is>
       </c>
       <c r="B16" s="29" t="n">
-        <v>343605.581</v>
+        <v>343805.581</v>
       </c>
       <c r="C16" s="29" t="n">
         <v>348432.349</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>0.2481</v>
+        <v>0.2479</v>
       </c>
       <c r="E16" s="30" t="n">
         <v>0.1411</v>
@@ -3089,7 +3089,7 @@
         </is>
       </c>
       <c r="B17" s="29" t="n">
-        <v>361815.215</v>
+        <v>362015.215</v>
       </c>
       <c r="C17" s="29" t="n">
         <v>361644.71</v>
@@ -3114,7 +3114,7 @@
         <v>358755.982</v>
       </c>
       <c r="D18" s="30" t="n">
-        <v>0.1285</v>
+        <v>0.1279</v>
       </c>
       <c r="E18" s="30" t="n">
         <v>0.0296</v>
@@ -3133,7 +3133,7 @@
         <v>361776.9</v>
       </c>
       <c r="D19" s="30" t="n">
-        <v>0.182</v>
+        <v>0.1813</v>
       </c>
       <c r="E19" s="30" t="n">
         <v>0.0383</v>
@@ -3152,7 +3152,7 @@
         <v>392410.404</v>
       </c>
       <c r="D20" s="30" t="n">
-        <v>0.21</v>
+        <v>0.2093</v>
       </c>
       <c r="E20" s="30" t="n">
         <v>0.1262</v>
@@ -3279,13 +3279,13 @@
         </is>
       </c>
       <c r="B27" s="29" t="n">
-        <v>617924.5699999999</v>
+        <v>623324.5699999999</v>
       </c>
       <c r="C27" s="29" t="n">
         <v>646939.245</v>
       </c>
       <c r="D27" s="30" t="n">
-        <v>0.2057</v>
+        <v>0.2162</v>
       </c>
       <c r="E27" s="30" t="n">
         <v>0.1399</v>
@@ -3298,13 +3298,13 @@
         </is>
       </c>
       <c r="B28" s="29" t="n">
-        <v>623634.2709999999</v>
+        <v>630534.2709999999</v>
       </c>
       <c r="C28" s="29" t="n">
         <v>693564.9534999999</v>
       </c>
       <c r="D28" s="30" t="n">
-        <v>0.2168</v>
+        <v>0.2303</v>
       </c>
       <c r="E28" s="30" t="n">
         <v>0.222</v>
@@ -3317,13 +3317,13 @@
         </is>
       </c>
       <c r="B29" s="29" t="n">
-        <v>655007.208</v>
+        <v>661907.208</v>
       </c>
       <c r="C29" s="29" t="n">
         <v>705856.914</v>
       </c>
       <c r="D29" s="30" t="n">
-        <v>0.0503</v>
+        <v>0.0498</v>
       </c>
       <c r="E29" s="30" t="n">
         <v>0.0177</v>
@@ -3336,13 +3336,13 @@
         </is>
       </c>
       <c r="B30" s="29" t="n">
-        <v>700801.926</v>
+        <v>706201.926</v>
       </c>
       <c r="C30" s="29" t="n">
         <v>739872.9861999999</v>
       </c>
       <c r="D30" s="30" t="n">
-        <v>0.1237</v>
+        <v>0.12</v>
       </c>
       <c r="E30" s="30" t="n">
         <v>0.0668</v>
@@ -3361,7 +3361,7 @@
         <v>801598.9116000001</v>
       </c>
       <c r="D31" s="30" t="n">
-        <v>0.2124</v>
+        <v>0.1991</v>
       </c>
       <c r="E31" s="30" t="n">
         <v>0.1558</v>
@@ -3380,7 +3380,7 @@
         <v>875042.3212</v>
       </c>
       <c r="D32" s="30" t="n">
-        <v>0.214</v>
+        <v>0.2008</v>
       </c>
       <c r="E32" s="30" t="n">
         <v>0.2617</v>
@@ -5581,19 +5581,19 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>93573.522</v>
+        <v>200</v>
       </c>
       <c r="C4" s="13" t="n">
-        <v>79300.508</v>
+        <v>0</v>
       </c>
       <c r="D4" s="13" t="n">
-        <v>118208.799</v>
+        <v>0</v>
       </c>
       <c r="E4" s="13" t="n">
-        <v>85211.565</v>
+        <v>6900</v>
       </c>
       <c r="F4" s="13" t="n">
-        <v>97010.931</v>
+        <v>0</v>
       </c>
       <c r="G4" s="10">
         <f>F4*(1+'02_Assumptions'!G4)</f>

</xml_diff>

<commit_message>
Update all components to use QoQ quarterly growth rate for credit and funding history
</commit_message>
<xml_diff>
--- a/Bao cao/TCB/TCB_Model_2026-06.xlsx
+++ b/Bao cao/TCB/TCB_Model_2026-06.xlsx
@@ -2788,12 +2788,12 @@
       </c>
       <c r="D1" s="9" t="inlineStr">
         <is>
-          <t>Tăng trưởng Tín dụng YTD (%)</t>
+          <t>Tăng trưởng Tín dụng QoQ (%)</t>
         </is>
       </c>
       <c r="E1" s="9" t="inlineStr">
         <is>
-          <t>Tăng trưởng Huy động YTD (%)</t>
+          <t>Tăng trưởng Huy động QoQ (%)</t>
         </is>
       </c>
     </row>
@@ -2810,10 +2810,10 @@
         <v>205187.505</v>
       </c>
       <c r="D2" s="30" t="n">
-        <v>0</v>
+        <v>0.0032</v>
       </c>
       <c r="E2" s="30" t="n">
-        <v>0</v>
+        <v>0.0185</v>
       </c>
     </row>
     <row r="3">
@@ -2848,10 +2848,10 @@
         <v>214649.295</v>
       </c>
       <c r="D4" s="30" t="n">
-        <v>0.0561</v>
+        <v>-0.0137</v>
       </c>
       <c r="E4" s="30" t="n">
-        <v>0.0461</v>
+        <v>0.0181</v>
       </c>
     </row>
     <row r="5">
@@ -2886,10 +2886,10 @@
         <v>232904.78</v>
       </c>
       <c r="D6" s="30" t="n">
-        <v>0.1097</v>
+        <v>0.1142</v>
       </c>
       <c r="E6" s="30" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.0546</v>
       </c>
     </row>
     <row r="7">
@@ -2905,10 +2905,10 @@
         <v>233143.291</v>
       </c>
       <c r="D7" s="30" t="n">
-        <v>0.1877</v>
+        <v>0.0703</v>
       </c>
       <c r="E7" s="30" t="n">
-        <v>0.0862</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="8">
@@ -2924,10 +2924,10 @@
         <v>248757.395</v>
       </c>
       <c r="D8" s="30" t="n">
-        <v>0.2829</v>
+        <v>0.0801</v>
       </c>
       <c r="E8" s="30" t="n">
-        <v>0.1589</v>
+        <v>0.067</v>
       </c>
     </row>
     <row r="9">
@@ -2962,10 +2962,10 @@
         <v>273261.751</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.0015</v>
       </c>
       <c r="E10" s="30" t="n">
-        <v>0.09849999999999999</v>
+        <v>0.0819</v>
       </c>
     </row>
     <row r="11">
@@ -2981,10 +2981,10 @@
         <v>275357.326</v>
       </c>
       <c r="D11" s="30" t="n">
-        <v>0.0034</v>
+        <v>-0.0053</v>
       </c>
       <c r="E11" s="30" t="n">
-        <v>0.1069</v>
+        <v>0.0077</v>
       </c>
     </row>
     <row r="12">
@@ -3000,10 +3000,10 @@
         <v>305358.291</v>
       </c>
       <c r="D12" s="30" t="n">
-        <v>0.2079</v>
+        <v>0.2038</v>
       </c>
       <c r="E12" s="30" t="n">
-        <v>0.2275</v>
+        <v>0.109</v>
       </c>
     </row>
     <row r="13">
@@ -3038,10 +3038,10 @@
         <v>317012.396</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>0.1282</v>
+        <v>0.0572</v>
       </c>
       <c r="E14" s="30" t="n">
-        <v>0.0382</v>
+        <v>0.0113</v>
       </c>
     </row>
     <row r="15">
@@ -3057,10 +3057,10 @@
         <v>350378.727</v>
       </c>
       <c r="D15" s="30" t="n">
-        <v>0.1537</v>
+        <v>0.0227</v>
       </c>
       <c r="E15" s="30" t="n">
-        <v>0.1474</v>
+        <v>0.1053</v>
       </c>
     </row>
     <row r="16">
@@ -3076,10 +3076,10 @@
         <v>348432.349</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>0.2479</v>
+        <v>0.08160000000000001</v>
       </c>
       <c r="E16" s="30" t="n">
-        <v>0.1411</v>
+        <v>-0.005600000000000001</v>
       </c>
     </row>
     <row r="17">
@@ -3114,10 +3114,10 @@
         <v>358755.982</v>
       </c>
       <c r="D18" s="30" t="n">
-        <v>0.1279</v>
+        <v>0.0712</v>
       </c>
       <c r="E18" s="30" t="n">
-        <v>0.0296</v>
+        <v>-0.008</v>
       </c>
     </row>
     <row r="19">
@@ -3133,10 +3133,10 @@
         <v>361776.9</v>
       </c>
       <c r="D19" s="30" t="n">
-        <v>0.1813</v>
+        <v>0.0474</v>
       </c>
       <c r="E19" s="30" t="n">
-        <v>0.0383</v>
+        <v>0.008399999999999999</v>
       </c>
     </row>
     <row r="20">
@@ -3152,10 +3152,10 @@
         <v>392410.404</v>
       </c>
       <c r="D20" s="30" t="n">
-        <v>0.2093</v>
+        <v>0.0236</v>
       </c>
       <c r="E20" s="30" t="n">
-        <v>0.1262</v>
+        <v>0.08470000000000001</v>
       </c>
     </row>
     <row r="21">
@@ -3190,10 +3190,10 @@
         <v>460661.7626</v>
       </c>
       <c r="D22" s="30" t="n">
-        <v>0.1082</v>
+        <v>0.0013</v>
       </c>
       <c r="E22" s="30" t="n">
-        <v>0.1739</v>
+        <v>0.0044</v>
       </c>
     </row>
     <row r="23">
@@ -3209,10 +3209,10 @@
         <v>496063.26375</v>
       </c>
       <c r="D23" s="30" t="n">
-        <v>0.1295</v>
+        <v>0.0192</v>
       </c>
       <c r="E23" s="30" t="n">
-        <v>0.2641</v>
+        <v>0.07679999999999999</v>
       </c>
     </row>
     <row r="24">
@@ -3228,10 +3228,10 @@
         <v>567554.2774</v>
       </c>
       <c r="D24" s="30" t="n">
-        <v>0.2327</v>
+        <v>0.09140000000000001</v>
       </c>
       <c r="E24" s="30" t="n">
-        <v>0.4463</v>
+        <v>0.1441</v>
       </c>
     </row>
     <row r="25">
@@ -3266,10 +3266,10 @@
         <v>629851.1385</v>
       </c>
       <c r="D26" s="30" t="n">
-        <v>0.1409</v>
+        <v>0.0582</v>
       </c>
       <c r="E26" s="30" t="n">
-        <v>0.1098</v>
+        <v>0.0702</v>
       </c>
     </row>
     <row r="27">
@@ -3285,10 +3285,10 @@
         <v>646939.245</v>
       </c>
       <c r="D27" s="30" t="n">
-        <v>0.2162</v>
+        <v>0.066</v>
       </c>
       <c r="E27" s="30" t="n">
-        <v>0.1399</v>
+        <v>0.0271</v>
       </c>
     </row>
     <row r="28">
@@ -3304,10 +3304,10 @@
         <v>693564.9534999999</v>
       </c>
       <c r="D28" s="30" t="n">
-        <v>0.2303</v>
+        <v>0.0116</v>
       </c>
       <c r="E28" s="30" t="n">
-        <v>0.222</v>
+        <v>0.0721</v>
       </c>
     </row>
     <row r="29">
@@ -3342,10 +3342,10 @@
         <v>739872.9861999999</v>
       </c>
       <c r="D30" s="30" t="n">
-        <v>0.12</v>
+        <v>0.0669</v>
       </c>
       <c r="E30" s="30" t="n">
-        <v>0.0668</v>
+        <v>0.0482</v>
       </c>
     </row>
     <row r="31">
@@ -3361,10 +3361,10 @@
         <v>801598.9116000001</v>
       </c>
       <c r="D31" s="30" t="n">
-        <v>0.1991</v>
+        <v>0.0706</v>
       </c>
       <c r="E31" s="30" t="n">
-        <v>0.1558</v>
+        <v>0.0834</v>
       </c>
     </row>
     <row r="32">
@@ -3380,10 +3380,10 @@
         <v>875042.3212</v>
       </c>
       <c r="D32" s="30" t="n">
-        <v>0.2008</v>
+        <v>0.0014</v>
       </c>
       <c r="E32" s="30" t="n">
-        <v>0.2617</v>
+        <v>0.0916</v>
       </c>
     </row>
     <row r="33">

</xml_diff>

<commit_message>
feat: integrate dynamic concurrent peer benchmark update, add stacked area IEA chart, NII and NPL/LLR charts, insert sheet 15 in excel and page 4 in pdf
</commit_message>
<xml_diff>
--- a/Bao cao/TCB/TCB_Model_2026-06.xlsx
+++ b/Bao cao/TCB/TCB_Model_2026-06.xlsx
@@ -25,6 +25,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Summary_Snapshot" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_PE_PB_History" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Credit_Funding_Growth" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Peer_Benchmark" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -39,7 +40,7 @@
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -97,8 +98,14 @@
       <color rgb="00C00000"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <i val="1"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -123,6 +130,18 @@
         <bgColor rgb="00FFFF99"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -142,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -184,6 +203,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="11" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="11" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="1" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="1" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="1" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3410,6 +3437,669 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Ngân hàng</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>NPL (%)</t>
+        </is>
+      </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>NIM (%)</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>CASA (%)</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>ROE (%)</t>
+        </is>
+      </c>
+      <c r="F1" s="9" t="inlineStr">
+        <is>
+          <t>CIR (%)</t>
+        </is>
+      </c>
+      <c r="G1" s="9" t="inlineStr">
+        <is>
+          <t>P/B (x)</t>
+        </is>
+      </c>
+      <c r="H1" s="9" t="inlineStr">
+        <is>
+          <t>Tăng trưởng tín dụng (%)</t>
+        </is>
+      </c>
+      <c r="I1" s="9" t="inlineStr">
+        <is>
+          <t>Vốn hóa (tỷ VND)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="31" t="inlineStr">
+        <is>
+          <t>Trung bình ngành</t>
+        </is>
+      </c>
+      <c r="B2" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" s="32" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D2" s="32" t="n">
+        <v>20</v>
+      </c>
+      <c r="E2" s="32" t="n">
+        <v>15</v>
+      </c>
+      <c r="F2" s="32" t="n">
+        <v>35</v>
+      </c>
+      <c r="G2" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="I2" s="31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>VCB — Vietcombank</t>
+        </is>
+      </c>
+      <c r="B3" s="30" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C3" s="30" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="D3" s="30" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E3" s="30" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F3" s="30" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G3" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="30" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="I3" s="29" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="28" t="inlineStr">
+        <is>
+          <t>BID — BIDV</t>
+        </is>
+      </c>
+      <c r="B4" s="30" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C4" s="30" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="D4" s="30" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E4" s="30" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F4" s="30" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G4" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="30" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="I4" s="29" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t>CTG — VietinBank</t>
+        </is>
+      </c>
+      <c r="B5" s="30" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C5" s="30" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="D5" s="30" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E5" s="30" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F5" s="30" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G5" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="30" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="I5" s="29" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="35" t="inlineStr">
+        <is>
+          <t>TCB — Techcombank</t>
+        </is>
+      </c>
+      <c r="B6" s="36" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C6" s="36" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="D6" s="36" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E6" s="36" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F6" s="36" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G6" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="36" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="I6" s="38" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>MBB — MBBank</t>
+        </is>
+      </c>
+      <c r="B7" s="30" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C7" s="30" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="D7" s="30" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E7" s="30" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F7" s="30" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G7" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="30" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="I7" s="29" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="28" t="inlineStr">
+        <is>
+          <t>ACB — ACB</t>
+        </is>
+      </c>
+      <c r="B8" s="30" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C8" s="30" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="D8" s="30" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E8" s="30" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F8" s="30" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G8" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="30" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="I8" s="29" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="28" t="inlineStr">
+        <is>
+          <t>VIB — VIB</t>
+        </is>
+      </c>
+      <c r="B9" s="30" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C9" s="30" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="D9" s="30" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E9" s="30" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F9" s="30" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G9" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="30" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="I9" s="29" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="28" t="inlineStr">
+        <is>
+          <t>HDB — HDBank</t>
+        </is>
+      </c>
+      <c r="B10" s="30" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C10" s="30" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="D10" s="30" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E10" s="30" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F10" s="30" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G10" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="30" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="I10" s="29" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="28" t="inlineStr">
+        <is>
+          <t>STB — Sacombank</t>
+        </is>
+      </c>
+      <c r="B11" s="30" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C11" s="30" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="D11" s="30" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E11" s="30" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F11" s="30" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G11" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="30" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="I11" s="29" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="28" t="inlineStr">
+        <is>
+          <t>VPB — VPBank</t>
+        </is>
+      </c>
+      <c r="B12" s="30" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C12" s="30" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="D12" s="30" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E12" s="30" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F12" s="30" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G12" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="30" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="I12" s="29" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="28" t="inlineStr">
+        <is>
+          <t>TPB — TPBank</t>
+        </is>
+      </c>
+      <c r="B13" s="30" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C13" s="30" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="D13" s="30" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E13" s="30" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F13" s="30" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G13" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="30" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="I13" s="29" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="28" t="inlineStr">
+        <is>
+          <t>MSB — MSB</t>
+        </is>
+      </c>
+      <c r="B14" s="30" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C14" s="30" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="D14" s="30" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E14" s="30" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F14" s="30" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G14" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="30" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="I14" s="29" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="28" t="inlineStr">
+        <is>
+          <t>EIB — Eximbank</t>
+        </is>
+      </c>
+      <c r="B15" s="30" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C15" s="30" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="D15" s="30" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E15" s="30" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F15" s="30" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G15" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="30" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="I15" s="29" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="28" t="inlineStr">
+        <is>
+          <t>LPB — LienVietPostBank</t>
+        </is>
+      </c>
+      <c r="B16" s="30" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C16" s="30" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="D16" s="30" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E16" s="30" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F16" s="30" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G16" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" s="30" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="I16" s="29" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="28" t="inlineStr">
+        <is>
+          <t>SHB — SHB</t>
+        </is>
+      </c>
+      <c r="B17" s="30" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C17" s="30" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="D17" s="30" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E17" s="30" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F17" s="30" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G17" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="30" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="I17" s="29" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="28" t="inlineStr">
+        <is>
+          <t>OCB — OCB</t>
+        </is>
+      </c>
+      <c r="B18" s="30" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C18" s="30" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="D18" s="30" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E18" s="30" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F18" s="30" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G18" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="30" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="I18" s="29" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="28" t="inlineStr">
+        <is>
+          <t>BAB — BacABank</t>
+        </is>
+      </c>
+      <c r="B19" s="30" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C19" s="30" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="D19" s="30" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E19" s="30" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F19" s="30" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G19" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="30" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="I19" s="29" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="28" t="inlineStr">
+        <is>
+          <t>NAB — NamABank</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C20" s="30" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="D20" s="30" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E20" s="30" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F20" s="30" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G20" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="30" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="I20" s="29" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
fix: correct share count keys for market cap calculations and update data registry and reports for VIB and TCB
</commit_message>
<xml_diff>
--- a/Bao cao/TCB/TCB_Model_2026-06.xlsx
+++ b/Bao cao/TCB/TCB_Model_2026-06.xlsx
@@ -3511,25 +3511,25 @@
         </is>
       </c>
       <c r="B2" s="32" t="n">
-        <v>2</v>
+        <v>2.385</v>
       </c>
       <c r="C2" s="32" t="n">
-        <v>3.5</v>
+        <v>4.357222222222222</v>
       </c>
       <c r="D2" s="32" t="n">
-        <v>20</v>
+        <v>16.84888888888889</v>
       </c>
       <c r="E2" s="32" t="n">
-        <v>15</v>
+        <v>15.58666666666667</v>
       </c>
       <c r="F2" s="32" t="n">
-        <v>35</v>
+        <v>33.94777777777777</v>
       </c>
       <c r="G2" s="33" t="n">
         <v>1</v>
       </c>
       <c r="H2" s="32" t="n">
-        <v>12</v>
+        <v>3.509444444444445</v>
       </c>
       <c r="I2" s="31" t="inlineStr">
         <is>
@@ -3544,28 +3544,28 @@
         </is>
       </c>
       <c r="B3" s="30" t="n">
-        <v>0.02</v>
+        <v>0.0063</v>
       </c>
       <c r="C3" s="30" t="n">
-        <v>0.035</v>
+        <v>0.0409</v>
       </c>
       <c r="D3" s="30" t="n">
-        <v>0.2</v>
+        <v>0.3255</v>
       </c>
       <c r="E3" s="30" t="n">
-        <v>0.15</v>
+        <v>0.1617</v>
       </c>
       <c r="F3" s="30" t="n">
-        <v>0.35</v>
+        <v>0.325</v>
       </c>
       <c r="G3" s="34" t="n">
         <v>1</v>
       </c>
       <c r="H3" s="30" t="n">
-        <v>0.12</v>
+        <v>0.0478</v>
       </c>
       <c r="I3" s="29" t="n">
-        <v>50000</v>
+        <v>513038.4507716</v>
       </c>
     </row>
     <row r="4">
@@ -3575,28 +3575,28 @@
         </is>
       </c>
       <c r="B4" s="30" t="n">
-        <v>0.02</v>
+        <v>0.0178</v>
       </c>
       <c r="C4" s="30" t="n">
-        <v>0.035</v>
+        <v>0.0263</v>
       </c>
       <c r="D4" s="30" t="n">
-        <v>0.2</v>
+        <v>0.1949</v>
       </c>
       <c r="E4" s="30" t="n">
-        <v>0.15</v>
+        <v>0.1443</v>
       </c>
       <c r="F4" s="30" t="n">
-        <v>0.35</v>
+        <v>0.3202</v>
       </c>
       <c r="G4" s="34" t="n">
         <v>1</v>
       </c>
       <c r="H4" s="30" t="n">
-        <v>0.12</v>
+        <v>0.0233</v>
       </c>
       <c r="I4" s="29" t="n">
-        <v>50000</v>
+        <v>303578.719257</v>
       </c>
     </row>
     <row r="5">
@@ -3606,28 +3606,28 @@
         </is>
       </c>
       <c r="B5" s="30" t="n">
-        <v>0.02</v>
+        <v>0.0103</v>
       </c>
       <c r="C5" s="30" t="n">
-        <v>0.035</v>
+        <v>0.0389</v>
       </c>
       <c r="D5" s="30" t="n">
-        <v>0.2</v>
+        <v>0.2408</v>
       </c>
       <c r="E5" s="30" t="n">
-        <v>0.15</v>
+        <v>0.1899</v>
       </c>
       <c r="F5" s="30" t="n">
-        <v>0.35</v>
+        <v>0.2494</v>
       </c>
       <c r="G5" s="34" t="n">
         <v>1</v>
       </c>
       <c r="H5" s="30" t="n">
-        <v>0.12</v>
+        <v>0.0187</v>
       </c>
       <c r="I5" s="29" t="n">
-        <v>50000</v>
+        <v>260969.3398032</v>
       </c>
     </row>
     <row r="6">
@@ -3637,28 +3637,28 @@
         </is>
       </c>
       <c r="B6" s="36" t="n">
-        <v>0.02</v>
+        <v>0.0111</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>0.035</v>
+        <v>0.04849999999999999</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>0.2</v>
+        <v>0.3145</v>
       </c>
       <c r="E6" s="36" t="n">
-        <v>0.15</v>
+        <v>0.1489</v>
       </c>
       <c r="F6" s="36" t="n">
-        <v>0.35</v>
+        <v>0.2829</v>
       </c>
       <c r="G6" s="37" t="n">
         <v>1</v>
       </c>
       <c r="H6" s="36" t="n">
-        <v>0.12</v>
+        <v>0.03759999999999999</v>
       </c>
       <c r="I6" s="38" t="n">
-        <v>50000</v>
+        <v>236680.4298276</v>
       </c>
     </row>
     <row r="7">
@@ -3668,28 +3668,28 @@
         </is>
       </c>
       <c r="B7" s="30" t="n">
-        <v>0.02</v>
+        <v>0.0144</v>
       </c>
       <c r="C7" s="30" t="n">
-        <v>0.035</v>
+        <v>0.0539</v>
       </c>
       <c r="D7" s="30" t="n">
-        <v>0.2</v>
+        <v>0.3227</v>
       </c>
       <c r="E7" s="30" t="n">
-        <v>0.15</v>
+        <v>0.2058</v>
       </c>
       <c r="F7" s="30" t="n">
-        <v>0.35</v>
+        <v>0.2494</v>
       </c>
       <c r="G7" s="34" t="n">
         <v>1</v>
       </c>
       <c r="H7" s="30" t="n">
-        <v>0.12</v>
+        <v>0.0327</v>
       </c>
       <c r="I7" s="29" t="n">
-        <v>50000</v>
+        <v>199361.24774775</v>
       </c>
     </row>
     <row r="8">
@@ -3699,28 +3699,28 @@
         </is>
       </c>
       <c r="B8" s="30" t="n">
-        <v>0.02</v>
+        <v>0.0098</v>
       </c>
       <c r="C8" s="30" t="n">
-        <v>0.035</v>
+        <v>0.0399</v>
       </c>
       <c r="D8" s="30" t="n">
-        <v>0.2</v>
+        <v>0.2123</v>
       </c>
       <c r="E8" s="30" t="n">
-        <v>0.15</v>
+        <v>0.175</v>
       </c>
       <c r="F8" s="30" t="n">
-        <v>0.35</v>
+        <v>0.3201</v>
       </c>
       <c r="G8" s="34" t="n">
         <v>1</v>
       </c>
       <c r="H8" s="30" t="n">
-        <v>0.12</v>
+        <v>0.0325</v>
       </c>
       <c r="I8" s="29" t="n">
-        <v>50000</v>
+        <v>131179.9362282</v>
       </c>
     </row>
     <row r="9">
@@ -3730,28 +3730,28 @@
         </is>
       </c>
       <c r="B9" s="30" t="n">
-        <v>0.02</v>
+        <v>0.0298</v>
       </c>
       <c r="C9" s="30" t="n">
-        <v>0.035</v>
+        <v>0.0424</v>
       </c>
       <c r="D9" s="30" t="n">
-        <v>0.2</v>
+        <v>0.1393</v>
       </c>
       <c r="E9" s="30" t="n">
-        <v>0.15</v>
+        <v>0.1824</v>
       </c>
       <c r="F9" s="30" t="n">
-        <v>0.35</v>
+        <v>0.3161</v>
       </c>
       <c r="G9" s="34" t="n">
         <v>1</v>
       </c>
       <c r="H9" s="30" t="n">
-        <v>0.12</v>
+        <v>0.0113</v>
       </c>
       <c r="I9" s="29" t="n">
-        <v>50000</v>
+        <v>54974.6922165</v>
       </c>
     </row>
     <row r="10">
@@ -3761,28 +3761,28 @@
         </is>
       </c>
       <c r="B10" s="30" t="n">
-        <v>0.02</v>
+        <v>0.0264</v>
       </c>
       <c r="C10" s="30" t="n">
-        <v>0.035</v>
+        <v>0.0572</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>0.2</v>
+        <v>0.1021</v>
       </c>
       <c r="E10" s="30" t="n">
-        <v>0.15</v>
+        <v>0.2357</v>
       </c>
       <c r="F10" s="30" t="n">
-        <v>0.35</v>
+        <v>0.2599</v>
       </c>
       <c r="G10" s="34" t="n">
         <v>1</v>
       </c>
       <c r="H10" s="30" t="n">
-        <v>0.12</v>
+        <v>0.1006</v>
       </c>
       <c r="I10" s="29" t="n">
-        <v>50000</v>
+        <v>127134.0186042</v>
       </c>
     </row>
     <row r="11">
@@ -3792,28 +3792,28 @@
         </is>
       </c>
       <c r="B11" s="30" t="n">
-        <v>0.02</v>
+        <v>0.06860000000000001</v>
       </c>
       <c r="C11" s="30" t="n">
-        <v>0.035</v>
+        <v>0.04</v>
       </c>
       <c r="D11" s="30" t="n">
-        <v>0.2</v>
+        <v>0.1592</v>
       </c>
       <c r="E11" s="30" t="n">
-        <v>0.15</v>
+        <v>0.1031</v>
       </c>
       <c r="F11" s="30" t="n">
-        <v>0.35</v>
+        <v>0.4521</v>
       </c>
       <c r="G11" s="34" t="n">
         <v>1</v>
       </c>
       <c r="H11" s="30" t="n">
-        <v>0.12</v>
+        <v>-0.0024</v>
       </c>
       <c r="I11" s="29" t="n">
-        <v>50000</v>
+        <v>138940.3982692</v>
       </c>
     </row>
     <row r="12">
@@ -3823,28 +3823,28 @@
         </is>
       </c>
       <c r="B12" s="30" t="n">
-        <v>0.02</v>
+        <v>0.0365</v>
       </c>
       <c r="C12" s="30" t="n">
-        <v>0.035</v>
+        <v>0.0664</v>
       </c>
       <c r="D12" s="30" t="n">
-        <v>0.2</v>
+        <v>0.1309</v>
       </c>
       <c r="E12" s="30" t="n">
-        <v>0.15</v>
+        <v>0.1357</v>
       </c>
       <c r="F12" s="30" t="n">
-        <v>0.35</v>
+        <v>0.2169</v>
       </c>
       <c r="G12" s="34" t="n">
         <v>1</v>
       </c>
       <c r="H12" s="30" t="n">
-        <v>0.12</v>
+        <v>0.1023</v>
       </c>
       <c r="I12" s="29" t="n">
-        <v>50000</v>
+        <v>212232.45632675</v>
       </c>
     </row>
     <row r="13">
@@ -3854,28 +3854,28 @@
         </is>
       </c>
       <c r="B13" s="30" t="n">
-        <v>0.02</v>
+        <v>0.0219</v>
       </c>
       <c r="C13" s="30" t="n">
-        <v>0.035</v>
+        <v>0.0443</v>
       </c>
       <c r="D13" s="30" t="n">
-        <v>0.2</v>
+        <v>0.1745</v>
       </c>
       <c r="E13" s="30" t="n">
-        <v>0.15</v>
+        <v>0.1401</v>
       </c>
       <c r="F13" s="30" t="n">
-        <v>0.35</v>
+        <v>0.4585</v>
       </c>
       <c r="G13" s="34" t="n">
         <v>1</v>
       </c>
       <c r="H13" s="30" t="n">
-        <v>0.12</v>
+        <v>0.0326</v>
       </c>
       <c r="I13" s="29" t="n">
-        <v>50000</v>
+        <v>44662.1546553</v>
       </c>
     </row>
     <row r="14">
@@ -3885,28 +3885,28 @@
         </is>
       </c>
       <c r="B14" s="30" t="n">
-        <v>0.02</v>
+        <v>0.027</v>
       </c>
       <c r="C14" s="30" t="n">
-        <v>0.035</v>
+        <v>0.0604</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>0.2</v>
+        <v>0.2551</v>
       </c>
       <c r="E14" s="30" t="n">
-        <v>0.15</v>
+        <v>0.1377</v>
       </c>
       <c r="F14" s="30" t="n">
-        <v>0.35</v>
+        <v>0.3451</v>
       </c>
       <c r="G14" s="34" t="n">
         <v>1</v>
       </c>
       <c r="H14" s="30" t="n">
-        <v>0.12</v>
+        <v>0.0464</v>
       </c>
       <c r="I14" s="29" t="n">
-        <v>50000</v>
+        <v>49608</v>
       </c>
     </row>
     <row r="15">
@@ -3916,28 +3916,28 @@
         </is>
       </c>
       <c r="B15" s="30" t="n">
-        <v>0.02</v>
+        <v>0.031</v>
       </c>
       <c r="C15" s="30" t="n">
-        <v>0.035</v>
+        <v>0.0295</v>
       </c>
       <c r="D15" s="30" t="n">
-        <v>0.2</v>
+        <v>0.1337</v>
       </c>
       <c r="E15" s="30" t="n">
-        <v>0.15</v>
+        <v>0.0407</v>
       </c>
       <c r="F15" s="30" t="n">
-        <v>0.35</v>
+        <v>0.5698</v>
       </c>
       <c r="G15" s="34" t="n">
         <v>1</v>
       </c>
       <c r="H15" s="30" t="n">
-        <v>0.12</v>
+        <v>0.0289</v>
       </c>
       <c r="I15" s="29" t="n">
-        <v>50000</v>
+        <v>38372.0445042</v>
       </c>
     </row>
     <row r="16">
@@ -3947,28 +3947,28 @@
         </is>
       </c>
       <c r="B16" s="30" t="n">
-        <v>0.02</v>
+        <v>0.0186</v>
       </c>
       <c r="C16" s="30" t="n">
-        <v>0.035</v>
+        <v>0.039</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>0.2</v>
+        <v>0.0649</v>
       </c>
       <c r="E16" s="30" t="n">
-        <v>0.15</v>
+        <v>0.1843</v>
       </c>
       <c r="F16" s="30" t="n">
-        <v>0.35</v>
+        <v>0.3014</v>
       </c>
       <c r="G16" s="34" t="n">
         <v>1</v>
       </c>
       <c r="H16" s="30" t="n">
-        <v>0.12</v>
+        <v>0.0284</v>
       </c>
       <c r="I16" s="29" t="n">
-        <v>50000</v>
+        <v>158325.9513</v>
       </c>
     </row>
     <row r="17">
@@ -3978,28 +3978,28 @@
         </is>
       </c>
       <c r="B17" s="30" t="n">
-        <v>0.02</v>
+        <v>0.0265</v>
       </c>
       <c r="C17" s="30" t="n">
-        <v>0.035</v>
+        <v>0.0357</v>
       </c>
       <c r="D17" s="30" t="n">
-        <v>0.2</v>
+        <v>0.0663</v>
       </c>
       <c r="E17" s="30" t="n">
-        <v>0.15</v>
+        <v>0.2078</v>
       </c>
       <c r="F17" s="30" t="n">
-        <v>0.35</v>
+        <v>0.1717</v>
       </c>
       <c r="G17" s="34" t="n">
         <v>1</v>
       </c>
       <c r="H17" s="30" t="n">
-        <v>0.12</v>
+        <v>0.0201</v>
       </c>
       <c r="I17" s="29" t="n">
-        <v>50000</v>
+        <v>72941.55738870001</v>
       </c>
     </row>
     <row r="18">
@@ -4009,28 +4009,28 @@
         </is>
       </c>
       <c r="B18" s="30" t="n">
-        <v>0.02</v>
+        <v>0.0359</v>
       </c>
       <c r="C18" s="30" t="n">
-        <v>0.035</v>
+        <v>0.0475</v>
       </c>
       <c r="D18" s="30" t="n">
-        <v>0.2</v>
+        <v>0.1067</v>
       </c>
       <c r="E18" s="30" t="n">
-        <v>0.15</v>
+        <v>0.1118</v>
       </c>
       <c r="F18" s="30" t="n">
-        <v>0.35</v>
+        <v>0.3709</v>
       </c>
       <c r="G18" s="34" t="n">
         <v>1</v>
       </c>
       <c r="H18" s="30" t="n">
-        <v>0.12</v>
+        <v>0.0272</v>
       </c>
       <c r="I18" s="29" t="n">
-        <v>50000</v>
+        <v>33820.7640068</v>
       </c>
     </row>
     <row r="19">
@@ -4040,28 +4040,28 @@
         </is>
       </c>
       <c r="B19" s="30" t="n">
-        <v>0.02</v>
+        <v>0.0191</v>
       </c>
       <c r="C19" s="30" t="n">
-        <v>0.035</v>
+        <v>0.0319</v>
       </c>
       <c r="D19" s="30" t="n">
-        <v>0.2</v>
+        <v>0.0305</v>
       </c>
       <c r="E19" s="30" t="n">
-        <v>0.15</v>
+        <v>0.0882</v>
       </c>
       <c r="F19" s="30" t="n">
-        <v>0.35</v>
+        <v>0.5122</v>
       </c>
       <c r="G19" s="34" t="n">
         <v>1</v>
       </c>
       <c r="H19" s="30" t="n">
-        <v>0.12</v>
+        <v>0.0246</v>
       </c>
       <c r="I19" s="29" t="n">
-        <v>50000</v>
+        <v>13715.3535204</v>
       </c>
     </row>
     <row r="20">
@@ -4071,28 +4071,28 @@
         </is>
       </c>
       <c r="B20" s="30" t="n">
-        <v>0.02</v>
+        <v>0.0183</v>
       </c>
       <c r="C20" s="30" t="n">
-        <v>0.035</v>
+        <v>0.0416</v>
       </c>
       <c r="D20" s="30" t="n">
-        <v>0.2</v>
+        <v>0.05889999999999999</v>
       </c>
       <c r="E20" s="30" t="n">
-        <v>0.15</v>
+        <v>0.2125</v>
       </c>
       <c r="F20" s="30" t="n">
-        <v>0.35</v>
+        <v>0.389</v>
       </c>
       <c r="G20" s="34" t="n">
         <v>1</v>
       </c>
       <c r="H20" s="30" t="n">
-        <v>0.12</v>
+        <v>0.0191</v>
       </c>
       <c r="I20" s="29" t="n">
-        <v>50000</v>
+        <v>28172.6307801</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: recalculate P/B dynamically using Market Cap / VCSH for all 18 peer banks on each stock analysis run, update reports for VIB and TCB
</commit_message>
<xml_diff>
--- a/Bao cao/TCB/TCB_Model_2026-06.xlsx
+++ b/Bao cao/TCB/TCB_Model_2026-06.xlsx
@@ -3526,7 +3526,7 @@
         <v>33.94777777777777</v>
       </c>
       <c r="G2" s="33" t="n">
-        <v>1</v>
+        <v>1.443888888888889</v>
       </c>
       <c r="H2" s="32" t="n">
         <v>3.509444444444445</v>
@@ -3559,7 +3559,7 @@
         <v>0.325</v>
       </c>
       <c r="G3" s="34" t="n">
-        <v>1</v>
+        <v>2.19</v>
       </c>
       <c r="H3" s="30" t="n">
         <v>0.0478</v>
@@ -3590,7 +3590,7 @@
         <v>0.3202</v>
       </c>
       <c r="G4" s="34" t="n">
-        <v>1</v>
+        <v>1.59</v>
       </c>
       <c r="H4" s="30" t="n">
         <v>0.0233</v>
@@ -3621,7 +3621,7 @@
         <v>0.2494</v>
       </c>
       <c r="G5" s="34" t="n">
-        <v>1</v>
+        <v>1.38</v>
       </c>
       <c r="H5" s="30" t="n">
         <v>0.0187</v>
@@ -3652,7 +3652,7 @@
         <v>0.2829</v>
       </c>
       <c r="G6" s="37" t="n">
-        <v>1</v>
+        <v>1.27</v>
       </c>
       <c r="H6" s="36" t="n">
         <v>0.03759999999999999</v>
@@ -3683,7 +3683,7 @@
         <v>0.2494</v>
       </c>
       <c r="G7" s="34" t="n">
-        <v>1</v>
+        <v>1.33</v>
       </c>
       <c r="H7" s="30" t="n">
         <v>0.0327</v>
@@ -3714,7 +3714,7 @@
         <v>0.3201</v>
       </c>
       <c r="G8" s="34" t="n">
-        <v>1</v>
+        <v>1.33</v>
       </c>
       <c r="H8" s="30" t="n">
         <v>0.0325</v>
@@ -3745,7 +3745,7 @@
         <v>0.3161</v>
       </c>
       <c r="G9" s="34" t="n">
-        <v>1</v>
+        <v>1.12</v>
       </c>
       <c r="H9" s="30" t="n">
         <v>0.0113</v>
@@ -3776,7 +3776,7 @@
         <v>0.2599</v>
       </c>
       <c r="G10" s="34" t="n">
-        <v>1</v>
+        <v>1.53</v>
       </c>
       <c r="H10" s="30" t="n">
         <v>0.1006</v>
@@ -3807,7 +3807,7 @@
         <v>0.4521</v>
       </c>
       <c r="G11" s="34" t="n">
-        <v>1</v>
+        <v>2.26</v>
       </c>
       <c r="H11" s="30" t="n">
         <v>-0.0024</v>
@@ -3838,7 +3838,7 @@
         <v>0.2169</v>
       </c>
       <c r="G12" s="34" t="n">
-        <v>1</v>
+        <v>1.14</v>
       </c>
       <c r="H12" s="30" t="n">
         <v>0.1023</v>
@@ -3869,7 +3869,7 @@
         <v>0.4585</v>
       </c>
       <c r="G13" s="34" t="n">
-        <v>1</v>
+        <v>0.93</v>
       </c>
       <c r="H13" s="30" t="n">
         <v>0.0326</v>
@@ -3900,7 +3900,7 @@
         <v>0.3451</v>
       </c>
       <c r="G14" s="34" t="n">
-        <v>1</v>
+        <v>1.13</v>
       </c>
       <c r="H14" s="30" t="n">
         <v>0.0464</v>
@@ -3931,7 +3931,7 @@
         <v>0.5698</v>
       </c>
       <c r="G15" s="34" t="n">
-        <v>1</v>
+        <v>1.45</v>
       </c>
       <c r="H15" s="30" t="n">
         <v>0.0289</v>
@@ -3962,7 +3962,7 @@
         <v>0.3014</v>
       </c>
       <c r="G16" s="34" t="n">
-        <v>1</v>
+        <v>3.2</v>
       </c>
       <c r="H16" s="30" t="n">
         <v>0.0284</v>
@@ -3993,7 +3993,7 @@
         <v>0.1717</v>
       </c>
       <c r="G17" s="34" t="n">
-        <v>1</v>
+        <v>1.02</v>
       </c>
       <c r="H17" s="30" t="n">
         <v>0.0201</v>
@@ -4024,7 +4024,7 @@
         <v>0.3709</v>
       </c>
       <c r="G18" s="34" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
       <c r="H18" s="30" t="n">
         <v>0.0272</v>
@@ -4055,7 +4055,7 @@
         <v>0.5122</v>
       </c>
       <c r="G19" s="34" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="H19" s="30" t="n">
         <v>0.0246</v>
@@ -4086,7 +4086,7 @@
         <v>0.389</v>
       </c>
       <c r="G20" s="34" t="n">
-        <v>1</v>
+        <v>1.14</v>
       </c>
       <c r="H20" s="30" t="n">
         <v>0.0191</v>

</xml_diff>

<commit_message>
feat: banking analysis v2 - quarterly charts, YTD credit growth, PB median fix, key metrics, AI commentary, contrasting colors, forecast table 2026F/2027F, skill docs updated
</commit_message>
<xml_diff>
--- a/Bao cao/TCB/TCB_Model_2026-06.xlsx
+++ b/Bao cao/TCB/TCB_Model_2026-06.xlsx
@@ -1,31 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_COE" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Cover" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Assumptions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Income_Model" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_PnL_Quarterly" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_PnL" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Balance_Sheet_Quarterly" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Balance_Sheet" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Ratios_Quarterly" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Ratios" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Valuation" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Sensitivity" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_PESTLE" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Leading_Indicators" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Investment_Thesis" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Summary_Snapshot" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_PE_PB_History" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_Credit_Funding_Growth" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_Peer_Benchmark" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="00_COE" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="01_Cover" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="02_Assumptions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="03_Income_Model" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="04_PnL_Quarterly" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="04_PnL" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="05_Balance_Sheet_Quarterly" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="05_Balance_Sheet" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="06_Ratios_Quarterly" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="06_Ratios" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="07_Valuation" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="08_Sensitivity" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="09_PESTLE" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="10_Leading_Indicators" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="11_Investment_Thesis" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="12_Summary_Snapshot" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="13_PE_PB_History" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="14_Credit_Funding_Growth" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="15_Peer_Benchmark" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1039,7 +1039,7 @@
         </is>
       </c>
       <c r="B6" s="14">
-        <f>'05_Balance_Sheet'!F10*1000000000/'02_Assumptions'!$B$3</f>
+        <f>'05_Balance_Sheet'!F10*1000000000/'02_Assumptions'!$F$3</f>
         <v/>
       </c>
     </row>
@@ -1061,7 +1061,7 @@
         </is>
       </c>
       <c r="B8" s="14">
-        <f>((D29*(1+B3)/(B2-B3))*D30)*0.5</f>
+        <f>(D29*(1+B3)/(B2-B3))*D30</f>
         <v/>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
         </is>
       </c>
       <c r="B13" s="16">
-        <f>PERCENTILE('13_PE_PB_History'!C21:C32, 0.25)</f>
+        <f>PERCENTILE('13_PE_PB_History'!C2:C32, 0.25)</f>
         <v/>
       </c>
       <c r="C13" s="17" t="inlineStr">
@@ -1117,7 +1117,7 @@
         </is>
       </c>
       <c r="B14" s="15">
-        <f>MEDIAN('13_PE_PB_History'!C21:C32)</f>
+        <f>MEDIAN('13_PE_PB_History'!C2:C32)</f>
         <v/>
       </c>
       <c r="C14" s="18" t="inlineStr">
@@ -1133,7 +1133,7 @@
         </is>
       </c>
       <c r="B15" s="19">
-        <f>PERCENTILE('13_PE_PB_History'!C21:C32, 0.75)</f>
+        <f>PERCENTILE('13_PE_PB_History'!C2:C32, 0.75)</f>
         <v/>
       </c>
       <c r="C15" s="20" t="inlineStr">
@@ -1380,19 +1380,19 @@
         <v>0.08</v>
       </c>
       <c r="B3" s="14" t="n">
-        <v>31535.18797399649</v>
+        <v>41880.25288588145</v>
       </c>
       <c r="C3" s="14" t="n">
-        <v>32641.84910125206</v>
+        <v>44336.07537899274</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>34191.17467940987</v>
+        <v>47774.22686934853</v>
       </c>
       <c r="E3" s="14" t="n">
-        <v>36515.16304664659</v>
+        <v>52931.45410488223</v>
       </c>
       <c r="F3" s="14" t="n">
-        <v>40388.47699204111</v>
+        <v>61526.83283077174</v>
       </c>
     </row>
     <row r="4">
@@ -1400,19 +1400,19 @@
         <v>0.1</v>
       </c>
       <c r="B4" s="14" t="n">
-        <v>29805.19904967938</v>
+        <v>38142.6019951838</v>
       </c>
       <c r="C4" s="14" t="n">
-        <v>30427.49014966673</v>
+        <v>39523.5454863515</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>31227.57870679332</v>
+        <v>41299.04426070997</v>
       </c>
       <c r="E4" s="14" t="n">
-        <v>32294.36344962878</v>
+        <v>43666.3759598546</v>
       </c>
       <c r="F4" s="14" t="n">
-        <v>33787.86208959842</v>
+        <v>46980.64033865709</v>
       </c>
     </row>
     <row r="5">
@@ -1420,19 +1420,19 @@
         <v>0.12</v>
       </c>
       <c r="B5" s="14" t="n">
-        <v>28691.30675930642</v>
+        <v>35766.15851902301</v>
       </c>
       <c r="C5" s="24" t="n">
-        <v>29084.20739003823</v>
+        <v>36638.05523857404</v>
       </c>
       <c r="D5" s="24" t="n">
-        <v>29564.41927204377</v>
+        <v>37703.70678469197</v>
       </c>
       <c r="E5" s="14" t="n">
-        <v>30164.6841245507</v>
+        <v>39035.7712173394</v>
       </c>
       <c r="F5" s="14" t="n">
-        <v>30936.45322063104</v>
+        <v>40748.42548788607</v>
       </c>
     </row>
     <row r="6">
@@ -1440,19 +1440,19 @@
         <v>0.14</v>
       </c>
       <c r="B6" s="14" t="n">
-        <v>27910.1467059452</v>
+        <v>34122.56762019797</v>
       </c>
       <c r="C6" s="24" t="n">
-        <v>28177.55640513715</v>
+        <v>34715.9839226033</v>
       </c>
       <c r="D6" s="24" t="n">
-        <v>28493.58604963673</v>
+        <v>35417.29409817323</v>
       </c>
       <c r="E6" s="14" t="n">
-        <v>28872.82162303623</v>
+        <v>36258.86630885715</v>
       </c>
       <c r="F6" s="14" t="n">
-        <v>29336.33176830227</v>
+        <v>37287.45456635972</v>
       </c>
     </row>
     <row r="7">
@@ -1460,19 +1460,19 @@
         <v>0.16</v>
       </c>
       <c r="B7" s="14" t="n">
-        <v>27329.3931569062</v>
+        <v>32918.60412272703</v>
       </c>
       <c r="C7" s="14" t="n">
-        <v>27521.24950928891</v>
+        <v>33344.35789144953</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>27742.62222357666</v>
+        <v>33835.6122399755</v>
       </c>
       <c r="E7" s="14" t="n">
-        <v>28000.8903902457</v>
+        <v>34408.7423132558</v>
       </c>
       <c r="F7" s="14" t="n">
-        <v>28306.11640540002</v>
+        <v>35086.07785440523</v>
       </c>
     </row>
   </sheetData>
@@ -1987,28 +1987,28 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>2342.138259321307</v>
+        <v>5245.180543828634</v>
       </c>
       <c r="C6" s="13" t="n">
-        <v>2599.182315001052</v>
+        <v>5810.361168285858</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>2313.583461303553</v>
+        <v>5164.17607576959</v>
       </c>
       <c r="E6" s="13" t="n">
-        <v>2767.53271288158</v>
+        <v>3080.051064624612</v>
       </c>
       <c r="F6" s="13" t="n">
-        <v>3300.988373289438</v>
+        <v>3662.65756380492</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>3874.048020649368</v>
+        <v>4298.503866354192</v>
       </c>
       <c r="H6" s="13" t="n">
-        <v>4584.964865186867</v>
+        <v>5087.311539519929</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>5264.448778375742</v>
+        <v>5841.242366499787</v>
       </c>
     </row>
     <row r="7">
@@ -2753,10 +2753,10 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>8.621472893978607</v>
+        <v>9.084766589499999</v>
       </c>
       <c r="C32" s="13" t="n">
-        <v>1.250761902115244</v>
+        <v>1.3379662441</v>
       </c>
       <c r="D32" s="10" t="n"/>
       <c r="E32" s="10" t="n"/>
@@ -2768,10 +2768,10 @@
         </is>
       </c>
       <c r="B34" s="26" t="n">
-        <v>8.70834359705</v>
+        <v>8.7821250597</v>
       </c>
       <c r="C34" s="27" t="n">
-        <v>1.272280842</v>
+        <v>1.327280517</v>
       </c>
       <c r="D34" s="28" t="n"/>
       <c r="E34" s="28" t="n"/>
@@ -4119,7 +4119,7 @@
     <row r="3">
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Ngân hàng TCB</t>
+          <t>Ngân hàng Thương mại Cổ phần Kỹ thương Việt Nam</t>
         </is>
       </c>
     </row>
@@ -4252,15 +4252,29 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>7862636600</v>
-      </c>
-      <c r="C3" s="10" t="n"/>
-      <c r="D3" s="10" t="n"/>
-      <c r="E3" s="10" t="n"/>
-      <c r="F3" s="10" t="n"/>
-      <c r="G3" s="10" t="n"/>
-      <c r="H3" s="10" t="n"/>
-      <c r="I3" s="10" t="n"/>
+        <v>3510914800</v>
+      </c>
+      <c r="C3" s="11" t="n">
+        <v>3517238500</v>
+      </c>
+      <c r="D3" s="11" t="n">
+        <v>3522510800</v>
+      </c>
+      <c r="E3" s="11" t="n">
+        <v>7064851700</v>
+      </c>
+      <c r="F3" s="11" t="n">
+        <v>7086240400</v>
+      </c>
+      <c r="G3" s="11" t="n">
+        <v>7086240400</v>
+      </c>
+      <c r="H3" s="11" t="n">
+        <v>7086240400</v>
+      </c>
+      <c r="I3" s="11" t="n">
+        <v>7086240400</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -4551,13 +4565,13 @@
       <c r="E15" s="10" t="n"/>
       <c r="F15" s="10" t="n"/>
       <c r="G15" s="13" t="n">
-        <v>1.45635777105</v>
+        <v>1.6737236525</v>
       </c>
       <c r="H15" s="13" t="n">
-        <v>1.45635777105</v>
+        <v>1.6737236525</v>
       </c>
       <c r="I15" s="13" t="n">
-        <v>1.45635777105</v>
+        <v>1.6737236525</v>
       </c>
     </row>
   </sheetData>
@@ -5726,30 +5740,30 @@
         </is>
       </c>
       <c r="B6" s="11" t="n">
-        <v>2342.138259321307</v>
+        <v>5245.180543828634</v>
       </c>
       <c r="C6" s="11" t="n">
-        <v>2599.182315001052</v>
+        <v>5810.361168285858</v>
       </c>
       <c r="D6" s="11" t="n">
-        <v>2313.583461303553</v>
+        <v>5164.17607576959</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>2767.53271288158</v>
+        <v>3080.051064624612</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>3300.988373289438</v>
+        <v>3662.65756380492</v>
       </c>
       <c r="G6" s="11">
-        <f>G5*1000000000/'02_Assumptions'!$B$3</f>
+        <f>G5*1000000000/'02_Assumptions'!G3</f>
         <v/>
       </c>
       <c r="H6" s="11">
-        <f>H5*1000000000/'02_Assumptions'!$B$3</f>
+        <f>H5*1000000000/'02_Assumptions'!H3</f>
         <v/>
       </c>
       <c r="I6" s="11">
-        <f>I5*1000000000/'02_Assumptions'!$B$3</f>
+        <f>I5*1000000000/'02_Assumptions'!I3</f>
         <v/>
       </c>
     </row>

</xml_diff>